<commit_message>
fix(docs): fix font encoding for Sheet 2 header row in General Notes Excel
</commit_message>
<xml_diff>
--- a/dist/General_Notes_Neo_Noi_Thep_TCVN_5574_2018.xlsx
+++ b/dist/General_Notes_Neo_Noi_Thep_TCVN_5574_2018.xlsx
@@ -144,13 +144,13 @@
     <t>QUY ĐỊNH CHI TIẾT VỀ NEO, NỐI VÀ UỐN MÓC CỐT THÉP (TCVN 5574:2018)</t>
   </si>
   <si>
-    <t>H梳죒g m沼쩭 / C梳쪀 ki沼뇆</t>
-  </si>
-  <si>
-    <t>N沼셢 dung quy 휃沼땙h k沼?thu梳춗 thi c척ng (General Notes)</t>
-  </si>
-  <si>
-    <t>C훱n c沼?ti챗u chu梳쯰</t>
+    <t>Hạng mục / Cấu kiện</t>
+  </si>
+  <si>
+    <t>Nội dung quy định kỹ thuật thi công (General Notes)</t>
+  </si>
+  <si>
+    <t>Căn cứ tiêu chuẩn</t>
   </si>
   <si>
     <t>1. NGUYÊN TẮC CHUNG</t>
@@ -1211,7 +1211,7 @@
         <v>360</v>
       </c>
       <c r="G15" s="9">
-        <v>480</v>
+        <v>420</v>
       </c>
       <c r="H15" s="9">
         <v>480</v>

</xml_diff>

<commit_message>
feat(cad): add native AutoCAD DWG drawing for rebar anchorage and lap splice details (TCVN 5574:2018)
</commit_message>
<xml_diff>
--- a/dist/General_Notes_Neo_Noi_Thep_TCVN_5574_2018.xlsx
+++ b/dist/General_Notes_Neo_Noi_Thep_TCVN_5574_2018.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="c:\Users\BIM\Documents\Github\Tekla-Addin\dist\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\BIM\Documents\Github\Tekla-Addin\dist\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -339,18 +339,6 @@
   <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -380,6 +368,18 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -672,1138 +672,1138 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="35.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="4"/>
-      <c r="C1" s="4"/>
-      <c r="D1" s="4"/>
-      <c r="E1" s="4"/>
-      <c r="F1" s="4"/>
-      <c r="G1" s="4"/>
-      <c r="H1" s="4"/>
-      <c r="I1" s="4"/>
-      <c r="J1" s="4"/>
-      <c r="K1" s="4"/>
-      <c r="L1" s="4"/>
-      <c r="M1" s="4"/>
-      <c r="N1" s="4"/>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+      <c r="E1" s="14"/>
+      <c r="F1" s="14"/>
+      <c r="G1" s="14"/>
+      <c r="H1" s="14"/>
+      <c r="I1" s="14"/>
+      <c r="J1" s="14"/>
+      <c r="K1" s="14"/>
+      <c r="L1" s="14"/>
+      <c r="M1" s="14"/>
+      <c r="N1" s="14"/>
     </row>
     <row r="2" spans="1:14" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="5" t="s">
+      <c r="A2" s="15" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
-      <c r="H2" s="2"/>
-      <c r="I2" s="2"/>
-      <c r="J2" s="2"/>
-      <c r="K2" s="2"/>
-      <c r="L2" s="2"/>
-      <c r="M2" s="2"/>
-      <c r="N2" s="2"/>
+      <c r="B2" s="16"/>
+      <c r="C2" s="16"/>
+      <c r="D2" s="16"/>
+      <c r="E2" s="16"/>
+      <c r="F2" s="16"/>
+      <c r="G2" s="16"/>
+      <c r="H2" s="16"/>
+      <c r="I2" s="16"/>
+      <c r="J2" s="16"/>
+      <c r="K2" s="16"/>
+      <c r="L2" s="16"/>
+      <c r="M2" s="16"/>
+      <c r="N2" s="16"/>
     </row>
     <row r="4" spans="1:14" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="6" t="s">
+      <c r="A4" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="B4" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="C4" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="D4" s="6" t="s">
+      <c r="D4" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="6" t="s">
+      <c r="E4" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="F4" s="6" t="s">
+      <c r="F4" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="G4" s="6" t="s">
+      <c r="G4" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="H4" s="6" t="s">
+      <c r="H4" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="I4" s="6" t="s">
+      <c r="I4" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="J4" s="6" t="s">
+      <c r="J4" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="K4" s="6" t="s">
+      <c r="K4" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="L4" s="6" t="s">
+      <c r="L4" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="M4" s="6" t="s">
+      <c r="M4" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="N4" s="6" t="s">
+      <c r="N4" s="2" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="5" spans="1:14" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="10" t="s">
+      <c r="A5" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="B5" s="7" t="s">
+      <c r="B5" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="C5" s="8" t="s">
+      <c r="C5" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="D5" s="7" t="s">
+      <c r="D5" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="E5" s="9">
+      <c r="E5" s="5">
         <v>300</v>
       </c>
-      <c r="F5" s="9">
+      <c r="F5" s="5">
         <v>360</v>
       </c>
-      <c r="G5" s="9">
+      <c r="G5" s="5">
         <v>420</v>
       </c>
-      <c r="H5" s="9">
+      <c r="H5" s="5">
         <v>480</v>
       </c>
-      <c r="I5" s="9">
+      <c r="I5" s="5">
         <v>540</v>
       </c>
-      <c r="J5" s="9">
+      <c r="J5" s="5">
         <v>600</v>
       </c>
-      <c r="K5" s="9">
+      <c r="K5" s="5">
         <v>660</v>
       </c>
-      <c r="L5" s="9">
+      <c r="L5" s="5">
         <v>750</v>
       </c>
-      <c r="M5" s="9">
+      <c r="M5" s="5">
         <v>840</v>
       </c>
-      <c r="N5" s="9">
+      <c r="N5" s="5">
         <v>960</v>
       </c>
     </row>
     <row r="6" spans="1:14" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="10" t="s">
+      <c r="A6" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="B6" s="7" t="s">
+      <c r="B6" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="C6" s="8" t="s">
+      <c r="C6" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="D6" s="7" t="s">
+      <c r="D6" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="E6" s="9">
+      <c r="E6" s="5">
         <v>200</v>
       </c>
-      <c r="F6" s="9">
+      <c r="F6" s="5">
         <v>240</v>
       </c>
-      <c r="G6" s="9">
+      <c r="G6" s="5">
         <v>280</v>
       </c>
-      <c r="H6" s="9">
+      <c r="H6" s="5">
         <v>320</v>
       </c>
-      <c r="I6" s="9">
+      <c r="I6" s="5">
         <v>360</v>
       </c>
-      <c r="J6" s="9">
+      <c r="J6" s="5">
         <v>400</v>
       </c>
-      <c r="K6" s="9">
+      <c r="K6" s="5">
         <v>440</v>
       </c>
-      <c r="L6" s="9">
+      <c r="L6" s="5">
         <v>500</v>
       </c>
-      <c r="M6" s="9">
+      <c r="M6" s="5">
         <v>560</v>
       </c>
-      <c r="N6" s="9">
+      <c r="N6" s="5">
         <v>640</v>
       </c>
     </row>
     <row r="7" spans="1:14" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="10" t="s">
+      <c r="A7" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="B7" s="7" t="s">
+      <c r="B7" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="C7" s="8" t="s">
+      <c r="C7" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="D7" s="7" t="s">
+      <c r="D7" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="E7" s="9">
+      <c r="E7" s="5">
         <v>350</v>
       </c>
-      <c r="F7" s="9">
+      <c r="F7" s="5">
         <v>420</v>
       </c>
-      <c r="G7" s="9">
+      <c r="G7" s="5">
         <v>490</v>
       </c>
-      <c r="H7" s="9">
+      <c r="H7" s="5">
         <v>560</v>
       </c>
-      <c r="I7" s="9">
+      <c r="I7" s="5">
         <v>630</v>
       </c>
-      <c r="J7" s="9">
+      <c r="J7" s="5">
         <v>700</v>
       </c>
-      <c r="K7" s="9">
+      <c r="K7" s="5">
         <v>770</v>
       </c>
-      <c r="L7" s="9">
+      <c r="L7" s="5">
         <v>880</v>
       </c>
-      <c r="M7" s="9">
+      <c r="M7" s="5">
         <v>980</v>
       </c>
-      <c r="N7" s="9">
+      <c r="N7" s="5">
         <v>1120</v>
       </c>
     </row>
     <row r="8" spans="1:14" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="10" t="s">
+      <c r="A8" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="B8" s="7" t="s">
+      <c r="B8" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="C8" s="8" t="s">
+      <c r="C8" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="D8" s="7" t="s">
+      <c r="D8" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="E8" s="9">
+      <c r="E8" s="5">
         <v>250</v>
       </c>
-      <c r="F8" s="9">
+      <c r="F8" s="5">
         <v>300</v>
       </c>
-      <c r="G8" s="9">
+      <c r="G8" s="5">
         <v>350</v>
       </c>
-      <c r="H8" s="9">
+      <c r="H8" s="5">
         <v>400</v>
       </c>
-      <c r="I8" s="9">
+      <c r="I8" s="5">
         <v>450</v>
       </c>
-      <c r="J8" s="9">
+      <c r="J8" s="5">
         <v>500</v>
       </c>
-      <c r="K8" s="9">
+      <c r="K8" s="5">
         <v>550</v>
       </c>
-      <c r="L8" s="9">
+      <c r="L8" s="5">
         <v>630</v>
       </c>
-      <c r="M8" s="9">
+      <c r="M8" s="5">
         <v>700</v>
       </c>
-      <c r="N8" s="9">
+      <c r="N8" s="5">
         <v>800</v>
       </c>
     </row>
     <row r="9" spans="1:14" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="11" t="s">
+      <c r="A9" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="B9" s="7" t="s">
+      <c r="B9" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="C9" s="8" t="s">
+      <c r="C9" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="D9" s="7" t="s">
+      <c r="D9" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="E9" s="9">
+      <c r="E9" s="5">
         <v>350</v>
       </c>
-      <c r="F9" s="9">
+      <c r="F9" s="5">
         <v>420</v>
       </c>
-      <c r="G9" s="9">
+      <c r="G9" s="5">
         <v>490</v>
       </c>
-      <c r="H9" s="9">
+      <c r="H9" s="5">
         <v>560</v>
       </c>
-      <c r="I9" s="9">
+      <c r="I9" s="5">
         <v>630</v>
       </c>
-      <c r="J9" s="9">
+      <c r="J9" s="5">
         <v>700</v>
       </c>
-      <c r="K9" s="9">
+      <c r="K9" s="5">
         <v>770</v>
       </c>
-      <c r="L9" s="9">
+      <c r="L9" s="5">
         <v>880</v>
       </c>
-      <c r="M9" s="9">
+      <c r="M9" s="5">
         <v>980</v>
       </c>
-      <c r="N9" s="9">
+      <c r="N9" s="5">
         <v>1120</v>
       </c>
     </row>
     <row r="10" spans="1:14" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="11" t="s">
+      <c r="A10" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="B10" s="7" t="s">
+      <c r="B10" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="C10" s="8" t="s">
+      <c r="C10" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="D10" s="7" t="s">
+      <c r="D10" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="E10" s="9">
+      <c r="E10" s="5">
         <v>250</v>
       </c>
-      <c r="F10" s="9">
+      <c r="F10" s="5">
         <v>300</v>
       </c>
-      <c r="G10" s="9">
+      <c r="G10" s="5">
         <v>350</v>
       </c>
-      <c r="H10" s="9">
+      <c r="H10" s="5">
         <v>400</v>
       </c>
-      <c r="I10" s="9">
+      <c r="I10" s="5">
         <v>450</v>
       </c>
-      <c r="J10" s="9">
+      <c r="J10" s="5">
         <v>500</v>
       </c>
-      <c r="K10" s="9">
+      <c r="K10" s="5">
         <v>550</v>
       </c>
-      <c r="L10" s="9">
+      <c r="L10" s="5">
         <v>630</v>
       </c>
-      <c r="M10" s="9">
+      <c r="M10" s="5">
         <v>700</v>
       </c>
-      <c r="N10" s="9">
+      <c r="N10" s="5">
         <v>800</v>
       </c>
     </row>
     <row r="11" spans="1:14" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="11" t="s">
+      <c r="A11" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="B11" s="7" t="s">
+      <c r="B11" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="C11" s="8" t="s">
+      <c r="C11" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="D11" s="7" t="s">
+      <c r="D11" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="E11" s="9">
+      <c r="E11" s="5">
         <v>400</v>
       </c>
-      <c r="F11" s="9">
+      <c r="F11" s="5">
         <v>480</v>
       </c>
-      <c r="G11" s="9">
+      <c r="G11" s="5">
         <v>560</v>
       </c>
-      <c r="H11" s="9">
+      <c r="H11" s="5">
         <v>640</v>
       </c>
-      <c r="I11" s="9">
+      <c r="I11" s="5">
         <v>720</v>
       </c>
-      <c r="J11" s="9">
+      <c r="J11" s="5">
         <v>800</v>
       </c>
-      <c r="K11" s="9">
+      <c r="K11" s="5">
         <v>880</v>
       </c>
-      <c r="L11" s="9">
+      <c r="L11" s="5">
         <v>1000</v>
       </c>
-      <c r="M11" s="9">
+      <c r="M11" s="5">
         <v>1120</v>
       </c>
-      <c r="N11" s="9">
+      <c r="N11" s="5">
         <v>1280</v>
       </c>
     </row>
     <row r="12" spans="1:14" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="11" t="s">
+      <c r="A12" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="B12" s="7" t="s">
+      <c r="B12" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="C12" s="8" t="s">
+      <c r="C12" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="D12" s="7" t="s">
+      <c r="D12" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="E12" s="9">
+      <c r="E12" s="5">
         <v>500</v>
       </c>
-      <c r="F12" s="9">
+      <c r="F12" s="5">
         <v>600</v>
       </c>
-      <c r="G12" s="9">
+      <c r="G12" s="5">
         <v>700</v>
       </c>
-      <c r="H12" s="9">
+      <c r="H12" s="5">
         <v>800</v>
       </c>
-      <c r="I12" s="9">
+      <c r="I12" s="5">
         <v>900</v>
       </c>
-      <c r="J12" s="9">
+      <c r="J12" s="5">
         <v>1000</v>
       </c>
-      <c r="K12" s="9">
+      <c r="K12" s="5">
         <v>1100</v>
       </c>
-      <c r="L12" s="9">
+      <c r="L12" s="5">
         <v>1250</v>
       </c>
-      <c r="M12" s="9">
+      <c r="M12" s="5">
         <v>1400</v>
       </c>
-      <c r="N12" s="9">
+      <c r="N12" s="5">
         <v>1600</v>
       </c>
     </row>
     <row r="13" spans="1:14" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="11" t="s">
+      <c r="A13" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="B13" s="7" t="s">
+      <c r="B13" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="C13" s="8" t="s">
+      <c r="C13" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="D13" s="7" t="s">
+      <c r="D13" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="E13" s="9">
+      <c r="E13" s="5">
         <v>300</v>
       </c>
-      <c r="F13" s="9">
+      <c r="F13" s="5">
         <v>360</v>
       </c>
-      <c r="G13" s="9">
+      <c r="G13" s="5">
         <v>420</v>
       </c>
-      <c r="H13" s="9">
+      <c r="H13" s="5">
         <v>480</v>
       </c>
-      <c r="I13" s="9">
+      <c r="I13" s="5">
         <v>540</v>
       </c>
-      <c r="J13" s="9">
+      <c r="J13" s="5">
         <v>600</v>
       </c>
-      <c r="K13" s="9">
+      <c r="K13" s="5">
         <v>660</v>
       </c>
-      <c r="L13" s="9">
+      <c r="L13" s="5">
         <v>750</v>
       </c>
-      <c r="M13" s="9">
+      <c r="M13" s="5">
         <v>840</v>
       </c>
-      <c r="N13" s="9">
+      <c r="N13" s="5">
         <v>960</v>
       </c>
     </row>
     <row r="14" spans="1:14" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="12" t="s">
+      <c r="A14" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="B14" s="7" t="s">
+      <c r="B14" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="C14" s="8" t="s">
+      <c r="C14" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="D14" s="7" t="s">
+      <c r="D14" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="E14" s="9">
+      <c r="E14" s="5">
         <v>400</v>
       </c>
-      <c r="F14" s="9">
+      <c r="F14" s="5">
         <v>480</v>
       </c>
-      <c r="G14" s="9">
+      <c r="G14" s="5">
         <v>560</v>
       </c>
-      <c r="H14" s="9">
+      <c r="H14" s="5">
         <v>640</v>
       </c>
-      <c r="I14" s="9">
+      <c r="I14" s="5">
         <v>720</v>
       </c>
-      <c r="J14" s="9">
+      <c r="J14" s="5">
         <v>800</v>
       </c>
-      <c r="K14" s="9">
+      <c r="K14" s="5">
         <v>880</v>
       </c>
-      <c r="L14" s="9">
+      <c r="L14" s="5">
         <v>1000</v>
       </c>
-      <c r="M14" s="9">
+      <c r="M14" s="5">
         <v>1120</v>
       </c>
-      <c r="N14" s="9">
+      <c r="N14" s="5">
         <v>1280</v>
       </c>
     </row>
     <row r="15" spans="1:14" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="12" t="s">
+      <c r="A15" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="B15" s="7" t="s">
+      <c r="B15" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="C15" s="8" t="s">
+      <c r="C15" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="D15" s="7" t="s">
+      <c r="D15" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="E15" s="9">
+      <c r="E15" s="5">
         <v>300</v>
       </c>
-      <c r="F15" s="9">
+      <c r="F15" s="5">
         <v>360</v>
       </c>
-      <c r="G15" s="9">
+      <c r="G15" s="5">
         <v>420</v>
       </c>
-      <c r="H15" s="9">
+      <c r="H15" s="5">
         <v>480</v>
       </c>
-      <c r="I15" s="9">
+      <c r="I15" s="5">
         <v>540</v>
       </c>
-      <c r="J15" s="9">
+      <c r="J15" s="5">
         <v>600</v>
       </c>
-      <c r="K15" s="9">
+      <c r="K15" s="5">
         <v>660</v>
       </c>
-      <c r="L15" s="9">
+      <c r="L15" s="5">
         <v>750</v>
       </c>
-      <c r="M15" s="9">
+      <c r="M15" s="5">
         <v>840</v>
       </c>
-      <c r="N15" s="9">
+      <c r="N15" s="5">
         <v>960</v>
       </c>
     </row>
     <row r="16" spans="1:14" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="12" t="s">
+      <c r="A16" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="B16" s="7" t="s">
+      <c r="B16" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="C16" s="8" t="s">
+      <c r="C16" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="D16" s="7" t="s">
+      <c r="D16" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="E16" s="9">
+      <c r="E16" s="5">
         <v>450</v>
       </c>
-      <c r="F16" s="9">
+      <c r="F16" s="5">
         <v>540</v>
       </c>
-      <c r="G16" s="9">
+      <c r="G16" s="5">
         <v>630</v>
       </c>
-      <c r="H16" s="9">
+      <c r="H16" s="5">
         <v>720</v>
       </c>
-      <c r="I16" s="9">
+      <c r="I16" s="5">
         <v>810</v>
       </c>
-      <c r="J16" s="9">
+      <c r="J16" s="5">
         <v>900</v>
       </c>
-      <c r="K16" s="9">
+      <c r="K16" s="5">
         <v>990</v>
       </c>
-      <c r="L16" s="9">
+      <c r="L16" s="5">
         <v>1130</v>
       </c>
-      <c r="M16" s="9">
+      <c r="M16" s="5">
         <v>1260</v>
       </c>
-      <c r="N16" s="9">
+      <c r="N16" s="5">
         <v>1440</v>
       </c>
     </row>
     <row r="17" spans="1:14" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="12" t="s">
+      <c r="A17" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="B17" s="7" t="s">
+      <c r="B17" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="C17" s="8" t="s">
+      <c r="C17" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="D17" s="7" t="s">
+      <c r="D17" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="E17" s="9">
+      <c r="E17" s="5">
         <v>550</v>
       </c>
-      <c r="F17" s="9">
+      <c r="F17" s="5">
         <v>660</v>
       </c>
-      <c r="G17" s="9">
+      <c r="G17" s="5">
         <v>770</v>
       </c>
-      <c r="H17" s="9">
+      <c r="H17" s="5">
         <v>880</v>
       </c>
-      <c r="I17" s="9">
+      <c r="I17" s="5">
         <v>990</v>
       </c>
-      <c r="J17" s="9">
+      <c r="J17" s="5">
         <v>1100</v>
       </c>
-      <c r="K17" s="9">
+      <c r="K17" s="5">
         <v>1210</v>
       </c>
-      <c r="L17" s="9">
+      <c r="L17" s="5">
         <v>1380</v>
       </c>
-      <c r="M17" s="9">
+      <c r="M17" s="5">
         <v>1540</v>
       </c>
-      <c r="N17" s="9">
+      <c r="N17" s="5">
         <v>1760</v>
       </c>
     </row>
     <row r="18" spans="1:14" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="12" t="s">
+      <c r="A18" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="B18" s="7" t="s">
+      <c r="B18" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="C18" s="8" t="s">
+      <c r="C18" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="D18" s="7" t="s">
+      <c r="D18" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="E18" s="9">
+      <c r="E18" s="5">
         <v>350</v>
       </c>
-      <c r="F18" s="9">
+      <c r="F18" s="5">
         <v>420</v>
       </c>
-      <c r="G18" s="9">
+      <c r="G18" s="5">
         <v>490</v>
       </c>
-      <c r="H18" s="9">
+      <c r="H18" s="5">
         <v>560</v>
       </c>
-      <c r="I18" s="9">
+      <c r="I18" s="5">
         <v>630</v>
       </c>
-      <c r="J18" s="9">
+      <c r="J18" s="5">
         <v>700</v>
       </c>
-      <c r="K18" s="9">
+      <c r="K18" s="5">
         <v>770</v>
       </c>
-      <c r="L18" s="9">
+      <c r="L18" s="5">
         <v>880</v>
       </c>
-      <c r="M18" s="9">
+      <c r="M18" s="5">
         <v>980</v>
       </c>
-      <c r="N18" s="9">
+      <c r="N18" s="5">
         <v>1120</v>
       </c>
     </row>
     <row r="19" spans="1:14" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="12" t="s">
+      <c r="A19" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="B19" s="7" t="s">
+      <c r="B19" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="C19" s="8" t="s">
+      <c r="C19" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="D19" s="7" t="s">
+      <c r="D19" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="E19" s="9">
+      <c r="E19" s="5">
         <v>350</v>
       </c>
-      <c r="F19" s="9">
+      <c r="F19" s="5">
         <v>420</v>
       </c>
-      <c r="G19" s="9">
+      <c r="G19" s="5">
         <v>490</v>
       </c>
-      <c r="H19" s="9">
+      <c r="H19" s="5">
         <v>560</v>
       </c>
-      <c r="I19" s="9">
+      <c r="I19" s="5">
         <v>630</v>
       </c>
-      <c r="J19" s="9">
+      <c r="J19" s="5">
         <v>700</v>
       </c>
-      <c r="K19" s="9">
+      <c r="K19" s="5">
         <v>770</v>
       </c>
-      <c r="L19" s="9">
+      <c r="L19" s="5">
         <v>880</v>
       </c>
-      <c r="M19" s="9">
+      <c r="M19" s="5">
         <v>980</v>
       </c>
-      <c r="N19" s="9">
+      <c r="N19" s="5">
         <v>1120</v>
       </c>
     </row>
     <row r="20" spans="1:14" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="12" t="s">
+      <c r="A20" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="B20" s="7" t="s">
+      <c r="B20" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="C20" s="8" t="s">
+      <c r="C20" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="D20" s="7" t="s">
+      <c r="D20" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="E20" s="9">
+      <c r="E20" s="5">
         <v>250</v>
       </c>
-      <c r="F20" s="9">
+      <c r="F20" s="5">
         <v>300</v>
       </c>
-      <c r="G20" s="9">
+      <c r="G20" s="5">
         <v>350</v>
       </c>
-      <c r="H20" s="9">
+      <c r="H20" s="5">
         <v>400</v>
       </c>
-      <c r="I20" s="9">
+      <c r="I20" s="5">
         <v>450</v>
       </c>
-      <c r="J20" s="9">
+      <c r="J20" s="5">
         <v>500</v>
       </c>
-      <c r="K20" s="9">
+      <c r="K20" s="5">
         <v>550</v>
       </c>
-      <c r="L20" s="9">
+      <c r="L20" s="5">
         <v>630</v>
       </c>
-      <c r="M20" s="9">
+      <c r="M20" s="5">
         <v>700</v>
       </c>
-      <c r="N20" s="9">
+      <c r="N20" s="5">
         <v>800</v>
       </c>
     </row>
     <row r="21" spans="1:14" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="12" t="s">
+      <c r="A21" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="B21" s="7" t="s">
+      <c r="B21" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="C21" s="8" t="s">
+      <c r="C21" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="D21" s="7" t="s">
+      <c r="D21" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="E21" s="9">
+      <c r="E21" s="5">
         <v>400</v>
       </c>
-      <c r="F21" s="9">
+      <c r="F21" s="5">
         <v>480</v>
       </c>
-      <c r="G21" s="9">
+      <c r="G21" s="5">
         <v>560</v>
       </c>
-      <c r="H21" s="9">
+      <c r="H21" s="5">
         <v>640</v>
       </c>
-      <c r="I21" s="9">
+      <c r="I21" s="5">
         <v>720</v>
       </c>
-      <c r="J21" s="9">
+      <c r="J21" s="5">
         <v>800</v>
       </c>
-      <c r="K21" s="9">
+      <c r="K21" s="5">
         <v>880</v>
       </c>
-      <c r="L21" s="9">
+      <c r="L21" s="5">
         <v>1000</v>
       </c>
-      <c r="M21" s="9">
+      <c r="M21" s="5">
         <v>1120</v>
       </c>
-      <c r="N21" s="9">
+      <c r="N21" s="5">
         <v>1280</v>
       </c>
     </row>
     <row r="22" spans="1:14" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="12" t="s">
+      <c r="A22" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="B22" s="7" t="s">
+      <c r="B22" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="C22" s="8" t="s">
+      <c r="C22" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="D22" s="7" t="s">
+      <c r="D22" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="E22" s="9">
+      <c r="E22" s="5">
         <v>500</v>
       </c>
-      <c r="F22" s="9">
+      <c r="F22" s="5">
         <v>600</v>
       </c>
-      <c r="G22" s="9">
+      <c r="G22" s="5">
         <v>700</v>
       </c>
-      <c r="H22" s="9">
+      <c r="H22" s="5">
         <v>800</v>
       </c>
-      <c r="I22" s="9">
+      <c r="I22" s="5">
         <v>900</v>
       </c>
-      <c r="J22" s="9">
+      <c r="J22" s="5">
         <v>1000</v>
       </c>
-      <c r="K22" s="9">
+      <c r="K22" s="5">
         <v>1100</v>
       </c>
-      <c r="L22" s="9">
+      <c r="L22" s="5">
         <v>1250</v>
       </c>
-      <c r="M22" s="9">
+      <c r="M22" s="5">
         <v>1400</v>
       </c>
-      <c r="N22" s="9">
+      <c r="N22" s="5">
         <v>1600</v>
       </c>
     </row>
     <row r="23" spans="1:14" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="12" t="s">
+      <c r="A23" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="B23" s="7" t="s">
+      <c r="B23" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="C23" s="8" t="s">
+      <c r="C23" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="D23" s="7" t="s">
+      <c r="D23" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="E23" s="9">
+      <c r="E23" s="5">
         <v>300</v>
       </c>
-      <c r="F23" s="9">
+      <c r="F23" s="5">
         <v>360</v>
       </c>
-      <c r="G23" s="9">
+      <c r="G23" s="5">
         <v>420</v>
       </c>
-      <c r="H23" s="9">
+      <c r="H23" s="5">
         <v>480</v>
       </c>
-      <c r="I23" s="9">
+      <c r="I23" s="5">
         <v>540</v>
       </c>
-      <c r="J23" s="9">
+      <c r="J23" s="5">
         <v>600</v>
       </c>
-      <c r="K23" s="9">
+      <c r="K23" s="5">
         <v>660</v>
       </c>
-      <c r="L23" s="9">
+      <c r="L23" s="5">
         <v>750</v>
       </c>
-      <c r="M23" s="9">
+      <c r="M23" s="5">
         <v>840</v>
       </c>
-      <c r="N23" s="9">
+      <c r="N23" s="5">
         <v>960</v>
       </c>
     </row>
     <row r="24" spans="1:14" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="13" t="s">
+      <c r="A24" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="B24" s="7" t="s">
+      <c r="B24" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="C24" s="8" t="s">
+      <c r="C24" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="D24" s="7" t="s">
+      <c r="D24" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="E24" s="9">
+      <c r="E24" s="5">
         <v>450</v>
       </c>
-      <c r="F24" s="9">
+      <c r="F24" s="5">
         <v>540</v>
       </c>
-      <c r="G24" s="9">
+      <c r="G24" s="5">
         <v>630</v>
       </c>
-      <c r="H24" s="9">
+      <c r="H24" s="5">
         <v>720</v>
       </c>
-      <c r="I24" s="9">
+      <c r="I24" s="5">
         <v>810</v>
       </c>
-      <c r="J24" s="9">
+      <c r="J24" s="5">
         <v>900</v>
       </c>
-      <c r="K24" s="9">
+      <c r="K24" s="5">
         <v>990</v>
       </c>
-      <c r="L24" s="9">
+      <c r="L24" s="5">
         <v>1130</v>
       </c>
-      <c r="M24" s="9">
+      <c r="M24" s="5">
         <v>1260</v>
       </c>
-      <c r="N24" s="9">
+      <c r="N24" s="5">
         <v>1440</v>
       </c>
     </row>
     <row r="25" spans="1:14" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="13" t="s">
+      <c r="A25" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="B25" s="7" t="s">
+      <c r="B25" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="C25" s="8" t="s">
+      <c r="C25" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="D25" s="7" t="s">
+      <c r="D25" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="E25" s="9">
+      <c r="E25" s="5">
         <v>320</v>
       </c>
-      <c r="F25" s="9">
+      <c r="F25" s="5">
         <v>390</v>
       </c>
-      <c r="G25" s="9">
+      <c r="G25" s="5">
         <v>450</v>
       </c>
-      <c r="H25" s="9">
+      <c r="H25" s="5">
         <v>520</v>
       </c>
-      <c r="I25" s="9">
+      <c r="I25" s="5">
         <v>580</v>
       </c>
-      <c r="J25" s="9">
+      <c r="J25" s="5">
         <v>640</v>
       </c>
-      <c r="K25" s="9">
+      <c r="K25" s="5">
         <v>710</v>
       </c>
-      <c r="L25" s="9">
+      <c r="L25" s="5">
         <v>800</v>
       </c>
-      <c r="M25" s="9">
+      <c r="M25" s="5">
         <v>900</v>
       </c>
-      <c r="N25" s="9">
+      <c r="N25" s="5">
         <v>1030</v>
       </c>
     </row>
     <row r="26" spans="1:14" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="13" t="s">
+      <c r="A26" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="B26" s="7" t="s">
+      <c r="B26" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="C26" s="8" t="s">
+      <c r="C26" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="D26" s="7" t="s">
+      <c r="D26" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="E26" s="9">
+      <c r="E26" s="5">
         <v>500</v>
       </c>
-      <c r="F26" s="9">
+      <c r="F26" s="5">
         <v>600</v>
       </c>
-      <c r="G26" s="9">
+      <c r="G26" s="5">
         <v>700</v>
       </c>
-      <c r="H26" s="9">
+      <c r="H26" s="5">
         <v>800</v>
       </c>
-      <c r="I26" s="9">
+      <c r="I26" s="5">
         <v>900</v>
       </c>
-      <c r="J26" s="9">
+      <c r="J26" s="5">
         <v>1000</v>
       </c>
-      <c r="K26" s="9">
+      <c r="K26" s="5">
         <v>1100</v>
       </c>
-      <c r="L26" s="9">
+      <c r="L26" s="5">
         <v>1250</v>
       </c>
-      <c r="M26" s="9">
+      <c r="M26" s="5">
         <v>1400</v>
       </c>
-      <c r="N26" s="9">
+      <c r="N26" s="5">
         <v>1600</v>
       </c>
     </row>
     <row r="27" spans="1:14" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="13" t="s">
+      <c r="A27" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="B27" s="7" t="s">
+      <c r="B27" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="C27" s="8" t="s">
+      <c r="C27" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="D27" s="7" t="s">
+      <c r="D27" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="E27" s="9">
+      <c r="E27" s="5">
         <v>600</v>
       </c>
-      <c r="F27" s="9">
+      <c r="F27" s="5">
         <v>720</v>
       </c>
-      <c r="G27" s="9">
+      <c r="G27" s="5">
         <v>840</v>
       </c>
-      <c r="H27" s="9">
+      <c r="H27" s="5">
         <v>960</v>
       </c>
-      <c r="I27" s="9">
+      <c r="I27" s="5">
         <v>1080</v>
       </c>
-      <c r="J27" s="9">
+      <c r="J27" s="5">
         <v>1200</v>
       </c>
-      <c r="K27" s="9">
+      <c r="K27" s="5">
         <v>1320</v>
       </c>
-      <c r="L27" s="9">
+      <c r="L27" s="5">
         <v>1500</v>
       </c>
-      <c r="M27" s="9">
+      <c r="M27" s="5">
         <v>1680</v>
       </c>
-      <c r="N27" s="9">
+      <c r="N27" s="5">
         <v>1920</v>
       </c>
     </row>
     <row r="28" spans="1:14" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="13" t="s">
+      <c r="A28" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="B28" s="7" t="s">
+      <c r="B28" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="C28" s="8" t="s">
+      <c r="C28" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="D28" s="7" t="s">
+      <c r="D28" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="E28" s="9">
+      <c r="E28" s="5">
         <v>350</v>
       </c>
-      <c r="F28" s="9">
+      <c r="F28" s="5">
         <v>420</v>
       </c>
-      <c r="G28" s="9">
+      <c r="G28" s="5">
         <v>490</v>
       </c>
-      <c r="H28" s="9">
+      <c r="H28" s="5">
         <v>560</v>
       </c>
-      <c r="I28" s="9">
+      <c r="I28" s="5">
         <v>630</v>
       </c>
-      <c r="J28" s="9">
+      <c r="J28" s="5">
         <v>700</v>
       </c>
-      <c r="K28" s="9">
+      <c r="K28" s="5">
         <v>770</v>
       </c>
-      <c r="L28" s="9">
+      <c r="L28" s="5">
         <v>880</v>
       </c>
-      <c r="M28" s="9">
+      <c r="M28" s="5">
         <v>980</v>
       </c>
-      <c r="N28" s="9">
+      <c r="N28" s="5">
         <v>1120</v>
       </c>
     </row>
@@ -1822,174 +1822,174 @@
   <dimension ref="A1:C18"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="28.7109375" style="1" customWidth="1"/>
-    <col min="2" max="2" width="85.7109375" style="1" customWidth="1"/>
-    <col min="3" max="3" width="18.7109375" style="1" customWidth="1"/>
+    <col min="1" max="1" width="34.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="84.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="35.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="13" t="s">
         <v>38</v>
       </c>
-      <c r="B1" s="4"/>
-      <c r="C1" s="4"/>
-    </row>
-    <row r="3" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="6" t="s">
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="B3" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="C3" s="2" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="14" t="s">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" s="10" t="s">
         <v>42</v>
       </c>
-      <c r="B4" s="15" t="s">
+      <c r="B4" s="11" t="s">
         <v>43</v>
       </c>
-      <c r="C4" s="7" t="s">
+      <c r="C4" s="3" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="16"/>
-      <c r="B5" s="15" t="s">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" s="12"/>
+      <c r="B5" s="11" t="s">
         <v>45</v>
       </c>
-      <c r="C5" s="7" t="s">
+      <c r="C5" s="3" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="16"/>
-      <c r="B6" s="15" t="s">
+    <row r="6" spans="1:3" ht="28.5" x14ac:dyDescent="0.25">
+      <c r="A6" s="12"/>
+      <c r="B6" s="11" t="s">
         <v>46</v>
       </c>
-      <c r="C6" s="7" t="s">
+      <c r="C6" s="3" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="16"/>
-      <c r="B7" s="15" t="s">
+    <row r="7" spans="1:3" ht="28.5" x14ac:dyDescent="0.25">
+      <c r="A7" s="12"/>
+      <c r="B7" s="11" t="s">
         <v>47</v>
       </c>
-      <c r="C7" s="7" t="s">
+      <c r="C7" s="3" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="14" t="s">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="B8" s="15" t="s">
+      <c r="B8" s="11" t="s">
         <v>49</v>
       </c>
-      <c r="C8" s="7" t="s">
+      <c r="C8" s="3" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="16"/>
-      <c r="B9" s="15" t="s">
+    <row r="9" spans="1:3" ht="28.5" x14ac:dyDescent="0.25">
+      <c r="A9" s="12"/>
+      <c r="B9" s="11" t="s">
         <v>50</v>
       </c>
-      <c r="C9" s="7" t="s">
+      <c r="C9" s="3" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="16"/>
-      <c r="B10" s="15" t="s">
+    <row r="10" spans="1:3" ht="28.5" x14ac:dyDescent="0.25">
+      <c r="A10" s="12"/>
+      <c r="B10" s="11" t="s">
         <v>51</v>
       </c>
-      <c r="C10" s="7" t="s">
+      <c r="C10" s="3" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="14" t="s">
+    <row r="11" spans="1:3" ht="28.5" x14ac:dyDescent="0.25">
+      <c r="A11" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="B11" s="15" t="s">
+      <c r="B11" s="11" t="s">
         <v>53</v>
       </c>
-      <c r="C11" s="7" t="s">
+      <c r="C11" s="3" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="12" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="16"/>
-      <c r="B12" s="15" t="s">
+    <row r="12" spans="1:3" ht="28.5" x14ac:dyDescent="0.25">
+      <c r="A12" s="12"/>
+      <c r="B12" s="11" t="s">
         <v>54</v>
       </c>
-      <c r="C12" s="7" t="s">
+      <c r="C12" s="3" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="16"/>
-      <c r="B13" s="15" t="s">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" s="12"/>
+      <c r="B13" s="11" t="s">
         <v>55</v>
       </c>
-      <c r="C13" s="7" t="s">
+      <c r="C13" s="3" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="14" t="s">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="B14" s="15" t="s">
+      <c r="B14" s="11" t="s">
         <v>57</v>
       </c>
-      <c r="C14" s="7" t="s">
+      <c r="C14" s="3" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="16"/>
-      <c r="B15" s="15" t="s">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A15" s="12"/>
+      <c r="B15" s="11" t="s">
         <v>58</v>
       </c>
-      <c r="C15" s="7" t="s">
+      <c r="C15" s="3" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="14" t="s">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A16" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="B16" s="15" t="s">
+      <c r="B16" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="C16" s="7" t="s">
+      <c r="C16" s="3" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="17" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="16"/>
-      <c r="B17" s="15" t="s">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A17" s="12"/>
+      <c r="B17" s="11" t="s">
         <v>61</v>
       </c>
-      <c r="C17" s="7" t="s">
+      <c r="C17" s="3" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="18" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="14" t="s">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A18" s="10" t="s">
         <v>62</v>
       </c>
-      <c r="B18" s="15" t="s">
+      <c r="B18" s="11" t="s">
         <v>63</v>
       </c>
-      <c r="C18" s="7" t="s">
+      <c r="C18" s="3" t="s">
         <v>44</v>
       </c>
     </row>

</xml_diff>